<commit_message>
Refactor models (LASSO, MIQP, Layered) and rolling backtest metrics/plots end-to-end
</commit_message>
<xml_diff>
--- a/results/summaries/experiment_results.xlsx
+++ b/results/summaries/experiment_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H57"/>
+  <dimension ref="A1:N71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,30 +429,60 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>train_length_days</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>eval_length_days</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>TE_annual</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>TE_annual_oos</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>portfolio_return_oos</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>benchmark_return_oos</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>tracking_difference_oos</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
         <is>
           <t>asset_active_share</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>sector_active_share</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>diversification</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>bench_diversification</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>execution_time</t>
         </is>
@@ -468,22 +498,40 @@
         <v>50</v>
       </c>
       <c r="C2" t="n">
-        <v>0.02132739211383509</v>
+        <v>756</v>
       </c>
       <c r="D2" t="n">
-        <v>0.6913153828449551</v>
+        <v>63</v>
       </c>
       <c r="E2" t="n">
-        <v>0.50601210477286</v>
+        <v>0.02131236702790284</v>
       </c>
       <c r="F2" t="n">
-        <v>0.6090632099380749</v>
+        <v>0.02898214234766692</v>
       </c>
       <c r="G2" t="n">
-        <v>0.3508708418375058</v>
+        <v>-0.005879112526291919</v>
       </c>
       <c r="H2" t="n">
-        <v>0.06168913841247559</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.034815873619366</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.4942060616684135</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.1359003642914478</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.6380136713244314</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.1180713176727295</v>
       </c>
     </row>
     <row r="3">
@@ -496,22 +544,40 @@
         <v>50</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0271365237564941</v>
+        <v>756</v>
       </c>
       <c r="D3" t="n">
-        <v>0.7012445831090325</v>
+        <v>63</v>
       </c>
       <c r="E3" t="n">
-        <v>0.2964965660977287</v>
+        <v>0.02500316655006096</v>
       </c>
       <c r="F3" t="n">
-        <v>0.5041445828163511</v>
+        <v>0.03388903467396046</v>
       </c>
       <c r="G3" t="n">
-        <v>0.3508708418375058</v>
+        <v>-0.008027889650215503</v>
       </c>
       <c r="H3" t="n">
-        <v>0.1238131523132324</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.03266709649544242</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.4842793980716085</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.05085953840957792</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.6396434455480413</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0.1389052867889404</v>
       </c>
     </row>
     <row r="4">
@@ -524,22 +590,40 @@
         <v>50</v>
       </c>
       <c r="C4" t="n">
-        <v>0.02104488256544924</v>
+        <v>756</v>
       </c>
       <c r="D4" t="n">
-        <v>0.7036123372226935</v>
+        <v>63</v>
       </c>
       <c r="E4" t="n">
-        <v>0.4284220332503345</v>
+        <v>0.02169387123635353</v>
       </c>
       <c r="F4" t="n">
-        <v>0.5976567617031896</v>
+        <v>0.026053028624837</v>
       </c>
       <c r="G4" t="n">
-        <v>0.369191655658143</v>
+        <v>-0.0177153865229206</v>
       </c>
       <c r="H4" t="n">
-        <v>0.04848527908325195</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.02297959962273732</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.4828301137268606</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.1214098638172978</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.6151692954455764</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0.0971229076385498</v>
       </c>
     </row>
     <row r="5">
@@ -552,918 +636,1512 @@
         <v>50</v>
       </c>
       <c r="C5" t="n">
-        <v>0.02295768877130792</v>
+        <v>756</v>
       </c>
       <c r="D5" t="n">
-        <v>0.705752720160354</v>
+        <v>63</v>
       </c>
       <c r="E5" t="n">
-        <v>0.2974233651463912</v>
+        <v>0.02285392663485375</v>
       </c>
       <c r="F5" t="n">
-        <v>0.6023723244509257</v>
+        <v>0.0286234381882239</v>
       </c>
       <c r="G5" t="n">
-        <v>0.369191655658143</v>
+        <v>-0.01178011062610118</v>
       </c>
       <c r="H5" t="n">
-        <v>0.1418652534484863</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.02891487551955674</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.4700943310775579</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.05687763868654893</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.6266394109535378</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.1118667125701904</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>LASSO</t>
+          <t>Contribution</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>50</v>
       </c>
       <c r="C6" t="n">
-        <v>0.01610893619558706</v>
+        <v>756</v>
       </c>
       <c r="D6" t="n">
-        <v>0.7368122929633074</v>
+        <v>63</v>
       </c>
       <c r="E6" t="n">
-        <v>0.4689825652596311</v>
+        <v>0.04804421985537957</v>
       </c>
       <c r="F6" t="n">
-        <v>0.6927857430097154</v>
+        <v>0.06968957290161558</v>
       </c>
       <c r="G6" t="n">
-        <v>0.2955872750924631</v>
+        <v>-0.0854645442364943</v>
       </c>
       <c r="H6" t="n">
-        <v>17.08637046813965</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I6" t="n">
+        <v>-0.04476955809083638</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.7592358135327385</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.4543523978149131</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.2558058777334848</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.1111617088317871</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>LASSO_sector</t>
+          <t>Contribution_sector</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>50</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0208315975709712</v>
+        <v>756</v>
       </c>
       <c r="D7" t="n">
-        <v>0.7386580324017329</v>
+        <v>63</v>
       </c>
       <c r="E7" t="n">
-        <v>0.3371762710250908</v>
+        <v>0.04857872315200212</v>
       </c>
       <c r="F7" t="n">
-        <v>0.6314552426122937</v>
+        <v>0.07003815524207944</v>
       </c>
       <c r="G7" t="n">
-        <v>0.2955872750924631</v>
+        <v>-0.08185284612912191</v>
       </c>
       <c r="H7" t="n">
-        <v>15.78896737098694</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I7" t="n">
+        <v>-0.041157859983464</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.7590156186864467</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.4156477001576254</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.2657933890571471</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0.1388983726501465</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MIQP_Gurobi</t>
+          <t>LASSO</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>50</v>
       </c>
       <c r="C8" t="n">
-        <v>0.01411525497960927</v>
+        <v>756</v>
       </c>
       <c r="D8" t="n">
-        <v>0.7726211905514109</v>
+        <v>63</v>
       </c>
       <c r="E8" t="n">
-        <v>0.5202107518664896</v>
+        <v>0.04292448113283771</v>
       </c>
       <c r="F8" t="n">
-        <v>0.6883742206610257</v>
+        <v>0.06528321606545273</v>
       </c>
       <c r="G8" t="n">
-        <v>0.2771978865150995</v>
+        <v>-0.01007435532557299</v>
       </c>
       <c r="H8" t="n">
-        <v>120.15953540802</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.03062063082008493</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.7694970725485981</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.2428043788374786</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.4763180028520042</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N8" t="n">
+        <v>51.90961384773254</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>LASSO_sector</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>50</v>
       </c>
       <c r="C9" t="n">
-        <v>0.01803924077481981</v>
+        <v>756</v>
       </c>
       <c r="D9" t="n">
-        <v>0.8546635701175858</v>
+        <v>63</v>
       </c>
       <c r="E9" t="n">
-        <v>0.5739057748213736</v>
+        <v>0.05099373917383115</v>
       </c>
       <c r="F9" t="n">
-        <v>0.664552933019502</v>
+        <v>0.06942608734531903</v>
       </c>
       <c r="G9" t="n">
-        <v>0.2505862592431231</v>
+        <v>-0.01814008311369586</v>
       </c>
       <c r="H9" t="n">
-        <v>180.5208249092102</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.02255490303196206</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.7845216156938069</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.09464296749731671</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.296665550961844</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0.1806323528289795</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Stratified</t>
+          <t>MIQP_Gurobi</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="C10" t="n">
-        <v>0.01725544574176463</v>
+        <v>756</v>
       </c>
       <c r="D10" t="n">
-        <v>0.6692394421473364</v>
+        <v>63</v>
       </c>
       <c r="E10" t="n">
-        <v>0.4117177135987425</v>
+        <v>0.01581474911254654</v>
       </c>
       <c r="F10" t="n">
-        <v>0.4893667586145352</v>
+        <v>0.02422043894840394</v>
       </c>
       <c r="G10" t="n">
-        <v>0.2873881903474687</v>
+        <v>-0.03837159444646943</v>
       </c>
       <c r="H10" t="n">
-        <v>0.1040918827056885</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.002323391699188493</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.5745584265980928</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.1446836190406057</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.6915518306628172</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N10" t="n">
+        <v>9.29414963722229</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Stratified_sector</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="C11" t="n">
-        <v>0.02012448525716034</v>
+        <v>756</v>
       </c>
       <c r="D11" t="n">
-        <v>0.6827142959386945</v>
+        <v>63</v>
       </c>
       <c r="E11" t="n">
-        <v>0.2368744445242545</v>
+        <v>0.01661130167512207</v>
       </c>
       <c r="F11" t="n">
-        <v>0.4693665560260944</v>
+        <v>0.02898962307016937</v>
       </c>
       <c r="G11" t="n">
-        <v>0.2873881903474687</v>
+        <v>-0.02673154251822574</v>
       </c>
       <c r="H11" t="n">
-        <v>0.1591172218322754</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.01396344362743218</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.5564856452383627</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0.04534465218204952</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.7313081443430997</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N11" t="n">
+        <v>16.30779886245728</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MarketCap</t>
+          <t>Stratified</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>75</v>
       </c>
       <c r="C12" t="n">
-        <v>0.01636878437124328</v>
+        <v>756</v>
       </c>
       <c r="D12" t="n">
-        <v>0.6812047983248539</v>
+        <v>63</v>
       </c>
       <c r="E12" t="n">
-        <v>0.3616764667404703</v>
+        <v>0.01817504008309745</v>
       </c>
       <c r="F12" t="n">
-        <v>0.5069108527244929</v>
+        <v>0.02216775095952048</v>
       </c>
       <c r="G12" t="n">
-        <v>0.2972021335942128</v>
+        <v>-0.01094629490005572</v>
       </c>
       <c r="H12" t="n">
-        <v>0.1179962158203125</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.0297486912456022</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.4464955681411947</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0.1072437112953941</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0.5073563617317465</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0.1806328296661377</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MarketCap_sector</t>
+          <t>Stratified_sector</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>75</v>
       </c>
       <c r="C13" t="n">
-        <v>0.01804072566683999</v>
+        <v>756</v>
       </c>
       <c r="D13" t="n">
-        <v>0.6681226276927538</v>
+        <v>63</v>
       </c>
       <c r="E13" t="n">
-        <v>0.2576304288494076</v>
+        <v>0.01975672894792977</v>
       </c>
       <c r="F13" t="n">
-        <v>0.5217471154439376</v>
+        <v>0.02613222234590185</v>
       </c>
       <c r="G13" t="n">
-        <v>0.2972021335942128</v>
+        <v>-0.006247586299658936</v>
       </c>
       <c r="H13" t="n">
-        <v>0.1382942199707031</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.03444739984599898</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.4491827201308318</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0.0479226137345647</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0.5116218355232899</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0.3123724460601807</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>LASSO</t>
+          <t>MarketCap</t>
         </is>
       </c>
       <c r="B14" t="n">
         <v>75</v>
       </c>
       <c r="C14" t="n">
-        <v>0.01314719097360715</v>
+        <v>756</v>
       </c>
       <c r="D14" t="n">
-        <v>0.6786550010087292</v>
+        <v>63</v>
       </c>
       <c r="E14" t="n">
-        <v>0.3906306381831665</v>
+        <v>0.0172233752563646</v>
       </c>
       <c r="F14" t="n">
-        <v>0.5518746772357291</v>
+        <v>0.02159582865523145</v>
       </c>
       <c r="G14" t="n">
-        <v>0.2404134011143279</v>
+        <v>-0.0237591331893745</v>
       </c>
       <c r="H14" t="n">
-        <v>14.91643738746643</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0.01693585295628341</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.4441624451123459</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0.08932426565912144</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0.5164290344076855</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N14" t="n">
+        <v>0.1804742813110352</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>LASSO_sector</t>
+          <t>MarketCap_sector</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>75</v>
       </c>
       <c r="C15" t="n">
-        <v>0.01482732818038358</v>
+        <v>756</v>
       </c>
       <c r="D15" t="n">
-        <v>0.6989481768090229</v>
+        <v>63</v>
       </c>
       <c r="E15" t="n">
-        <v>0.2907811673284774</v>
+        <v>0.01835558703928705</v>
       </c>
       <c r="F15" t="n">
-        <v>0.5481402643855534</v>
+        <v>0.02529588461067509</v>
       </c>
       <c r="G15" t="n">
-        <v>0.2404134011143279</v>
+        <v>-0.01907234591301421</v>
       </c>
       <c r="H15" t="n">
-        <v>14.75696206092834</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0.02162264023264371</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.4348978054430426</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0.03480572137970461</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0.5319500984030796</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0.2154147624969482</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>MIQP_Gurobi</t>
+          <t>Contribution</t>
         </is>
       </c>
       <c r="B16" t="n">
         <v>75</v>
       </c>
       <c r="C16" t="n">
-        <v>0.01197009063453958</v>
+        <v>756</v>
       </c>
       <c r="D16" t="n">
-        <v>0.6960165198533568</v>
+        <v>63</v>
       </c>
       <c r="E16" t="n">
-        <v>0.4786676645725263</v>
+        <v>0.0401042423105733</v>
       </c>
       <c r="F16" t="n">
-        <v>0.5420214872552992</v>
+        <v>0.05745664726140903</v>
       </c>
       <c r="G16" t="n">
-        <v>0.2233204633499571</v>
+        <v>-0.06897921814764196</v>
       </c>
       <c r="H16" t="n">
-        <v>120.1823954582214</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I16" t="n">
+        <v>-0.02828423200198404</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0.6776848227326888</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0.4036394485184417</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0.2409402950879602</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0.1320981979370117</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Contribution_sector</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>75</v>
       </c>
       <c r="C17" t="n">
-        <v>0.01947211016040492</v>
+        <v>756</v>
       </c>
       <c r="D17" t="n">
-        <v>0.9126587852200667</v>
+        <v>63</v>
       </c>
       <c r="E17" t="n">
-        <v>0.6638958665407887</v>
+        <v>0.0512690802385035</v>
       </c>
       <c r="F17" t="n">
-        <v>0.446350466645802</v>
+        <v>0.05684809021629608</v>
       </c>
       <c r="G17" t="n">
-        <v>0.1725795756123575</v>
+        <v>-0.05883077812650805</v>
       </c>
       <c r="H17" t="n">
-        <v>180.9333746433258</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I17" t="n">
+        <v>-0.01813579198085014</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0.6919918953020296</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0.2252381632266012</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0.2077261416443149</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N17" t="n">
+        <v>0.2435076236724854</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Stratified</t>
+          <t>LASSO</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="C18" t="n">
-        <v>0.01506176046625738</v>
+        <v>756</v>
       </c>
       <c r="D18" t="n">
-        <v>0.6686428398962571</v>
+        <v>63</v>
       </c>
       <c r="E18" t="n">
-        <v>0.3541931149452805</v>
+        <v>0.03491879634723517</v>
       </c>
       <c r="F18" t="n">
-        <v>0.4163386386940464</v>
+        <v>0.05506913734470776</v>
       </c>
       <c r="G18" t="n">
-        <v>0.2446957006007452</v>
+        <v>-0.01119021164602174</v>
       </c>
       <c r="H18" t="n">
-        <v>0.3334910869598389</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0.02950477449963618</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0.7371014637880446</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0.2096098580287993</v>
+      </c>
+      <c r="L18" t="n">
+        <v>0.3781404364457404</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N18" t="n">
+        <v>5.513991594314575</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Stratified_sector</t>
+          <t>LASSO_sector</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="C19" t="n">
-        <v>0.01698793703917529</v>
+        <v>756</v>
       </c>
       <c r="D19" t="n">
-        <v>0.6557202769497823</v>
+        <v>63</v>
       </c>
       <c r="E19" t="n">
-        <v>0.2029118512119675</v>
+        <v>0.03901597982657801</v>
       </c>
       <c r="F19" t="n">
-        <v>0.4080795303224793</v>
+        <v>0.05853004662567624</v>
       </c>
       <c r="G19" t="n">
-        <v>0.2446957006007452</v>
+        <v>-0.01057464469454938</v>
       </c>
       <c r="H19" t="n">
-        <v>0.5533185005187988</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0.03012034145110853</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.7435097078104378</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0.05301954699551756</v>
+      </c>
+      <c r="L19" t="n">
+        <v>0.2981819276466509</v>
+      </c>
+      <c r="M19" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N19" t="n">
+        <v>0.249382495880127</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>MarketCap</t>
+          <t>MIQP_Gurobi</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="C20" t="n">
-        <v>0.01497297321457867</v>
+        <v>756</v>
       </c>
       <c r="D20" t="n">
-        <v>0.6702185283406162</v>
+        <v>63</v>
       </c>
       <c r="E20" t="n">
-        <v>0.3395164795184332</v>
+        <v>0.01502830510081263</v>
       </c>
       <c r="F20" t="n">
-        <v>0.4226919936934812</v>
+        <v>0.02829438826279432</v>
       </c>
       <c r="G20" t="n">
-        <v>0.2544962768168757</v>
+        <v>-0.03056007620060475</v>
       </c>
       <c r="H20" t="n">
-        <v>0.3091669082641602</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0.01013490994505317</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0.5312895549326705</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0.1247162014286616</v>
+      </c>
+      <c r="L20" t="n">
+        <v>0.5327237813105689</v>
+      </c>
+      <c r="M20" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N20" t="n">
+        <v>2.819449901580811</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>MarketCap_sector</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="C21" t="n">
-        <v>0.01665668665750786</v>
+        <v>756</v>
       </c>
       <c r="D21" t="n">
-        <v>0.6681822924756847</v>
+        <v>63</v>
       </c>
       <c r="E21" t="n">
-        <v>0.2144935634384789</v>
+        <v>0.01583740736728497</v>
       </c>
       <c r="F21" t="n">
-        <v>0.4287926885388598</v>
+        <v>0.02451049375072392</v>
       </c>
       <c r="G21" t="n">
-        <v>0.2544962768168757</v>
+        <v>-0.0149410431467133</v>
       </c>
       <c r="H21" t="n">
-        <v>0.5001308917999268</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0.02575394299894462</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0.522702581487811</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0.05158697725878233</v>
+      </c>
+      <c r="L21" t="n">
+        <v>0.5666134379886667</v>
+      </c>
+      <c r="M21" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N21" t="n">
+        <v>3.416355609893799</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>LASSO</t>
+          <t>Stratified</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>100</v>
       </c>
       <c r="C22" t="n">
-        <v>0.01158665418410423</v>
+        <v>756</v>
       </c>
       <c r="D22" t="n">
-        <v>0.6135868444672994</v>
+        <v>63</v>
       </c>
       <c r="E22" t="n">
-        <v>0.3818946541668555</v>
+        <v>0.01603377965231577</v>
       </c>
       <c r="F22" t="n">
-        <v>0.4592637098830412</v>
+        <v>0.01981600501157972</v>
       </c>
       <c r="G22" t="n">
-        <v>0.2036089060797628</v>
+        <v>-0.01508080430447789</v>
       </c>
       <c r="H22" t="n">
-        <v>51.29146218299866</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0.02561418184118003</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0.4307787526313216</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0.1092710401830551</v>
+      </c>
+      <c r="L22" t="n">
+        <v>0.4206098664835803</v>
+      </c>
+      <c r="M22" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N22" t="n">
+        <v>0.2982041835784912</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>LASSO_sector</t>
+          <t>Stratified_sector</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>100</v>
       </c>
       <c r="C23" t="n">
-        <v>0.01362508108942149</v>
+        <v>756</v>
       </c>
       <c r="D23" t="n">
-        <v>0.6613838522934271</v>
+        <v>63</v>
       </c>
       <c r="E23" t="n">
-        <v>0.2644535393623868</v>
+        <v>0.01733475701631171</v>
       </c>
       <c r="F23" t="n">
-        <v>0.4552521689535684</v>
+        <v>0.02412535766743224</v>
       </c>
       <c r="G23" t="n">
-        <v>0.2036089060797628</v>
+        <v>-0.0128879348057096</v>
       </c>
       <c r="H23" t="n">
-        <v>51.76880145072937</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0.02780705133994832</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0.4237962739086217</v>
+      </c>
+      <c r="K23" t="n">
+        <v>0.04316680737975165</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0.4238981694381027</v>
+      </c>
+      <c r="M23" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N23" t="n">
+        <v>0.4189271926879883</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>MIQP_Gurobi</t>
+          <t>MarketCap</t>
         </is>
       </c>
       <c r="B24" t="n">
         <v>100</v>
       </c>
       <c r="C24" t="n">
-        <v>0.01129035135926354</v>
+        <v>756</v>
       </c>
       <c r="D24" t="n">
-        <v>0.6227138489621634</v>
+        <v>63</v>
       </c>
       <c r="E24" t="n">
-        <v>0.3898545659465498</v>
+        <v>0.01599000440446517</v>
       </c>
       <c r="F24" t="n">
-        <v>0.4465022803468148</v>
+        <v>0.02050648830326909</v>
       </c>
       <c r="G24" t="n">
-        <v>0.1927195903111882</v>
+        <v>-0.02563740902483225</v>
       </c>
       <c r="H24" t="n">
-        <v>120.6076302528381</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0.01505757712082567</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0.4257400314658467</v>
+      </c>
+      <c r="K24" t="n">
+        <v>0.09972769090631624</v>
+      </c>
+      <c r="L24" t="n">
+        <v>0.4307344066497592</v>
+      </c>
+      <c r="M24" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N24" t="n">
+        <v>0.2453789710998535</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MarketCap_sector</t>
         </is>
       </c>
       <c r="B25" t="n">
         <v>100</v>
       </c>
       <c r="C25" t="n">
-        <v>0.01712000106873682</v>
+        <v>756</v>
       </c>
       <c r="D25" t="n">
-        <v>0.827210671061219</v>
+        <v>63</v>
       </c>
       <c r="E25" t="n">
-        <v>0.6019575115561845</v>
+        <v>0.01710500216100064</v>
       </c>
       <c r="F25" t="n">
-        <v>0.3957644963265497</v>
+        <v>0.02528421723869915</v>
       </c>
       <c r="G25" t="n">
-        <v>0.1391359685726343</v>
+        <v>-0.01959634403416377</v>
       </c>
       <c r="H25" t="n">
-        <v>181.4077596664429</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0.02109864211149415</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0.4200882689826037</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0.0344328493783411</v>
+      </c>
+      <c r="L25" t="n">
+        <v>0.4410908211079539</v>
+      </c>
+      <c r="M25" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N25" t="n">
+        <v>0.3817026615142822</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Stratified</t>
+          <t>Contribution</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>125</v>
+        <v>100</v>
       </c>
       <c r="C26" t="n">
-        <v>0.01400214232316054</v>
+        <v>756</v>
       </c>
       <c r="D26" t="n">
-        <v>0.6600755814217011</v>
+        <v>63</v>
       </c>
       <c r="E26" t="n">
-        <v>0.317135581494805</v>
+        <v>0.03370984321386537</v>
       </c>
       <c r="F26" t="n">
-        <v>0.3557474589711965</v>
+        <v>0.05777352448971823</v>
       </c>
       <c r="G26" t="n">
-        <v>0.2184407082810675</v>
+        <v>-0.07125115198482967</v>
       </c>
       <c r="H26" t="n">
-        <v>0.1456601619720459</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I26" t="n">
+        <v>-0.03055616583917176</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0.6521055351974528</v>
+      </c>
+      <c r="K26" t="n">
+        <v>0.342742995148346</v>
+      </c>
+      <c r="L26" t="n">
+        <v>0.2141477482507501</v>
+      </c>
+      <c r="M26" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N26" t="n">
+        <v>0.2156002521514893</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Stratified_sector</t>
+          <t>Contribution_sector</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>125</v>
+        <v>100</v>
       </c>
       <c r="C27" t="n">
-        <v>0.01590934467375354</v>
+        <v>756</v>
       </c>
       <c r="D27" t="n">
-        <v>0.6398741218349786</v>
+        <v>63</v>
       </c>
       <c r="E27" t="n">
-        <v>0.2028531442656915</v>
+        <v>0.04892275471902595</v>
       </c>
       <c r="F27" t="n">
-        <v>0.3561488174674483</v>
+        <v>0.06336608982036861</v>
       </c>
       <c r="G27" t="n">
-        <v>0.2184407082810675</v>
+        <v>-0.07052662721115199</v>
       </c>
       <c r="H27" t="n">
-        <v>0.2036259174346924</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I27" t="n">
+        <v>-0.02983164106549407</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0.7140105346023771</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0.1147599126238575</v>
+      </c>
+      <c r="L27" t="n">
+        <v>0.1679006501159293</v>
+      </c>
+      <c r="M27" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N27" t="n">
+        <v>0.3539962768554688</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>MarketCap</t>
+          <t>LASSO</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>125</v>
+        <v>100</v>
       </c>
       <c r="C28" t="n">
-        <v>0.01380088221120567</v>
+        <v>756</v>
       </c>
       <c r="D28" t="n">
-        <v>0.6520436490064297</v>
+        <v>63</v>
       </c>
       <c r="E28" t="n">
-        <v>0.3102689673470634</v>
+        <v>0.0321020417815254</v>
       </c>
       <c r="F28" t="n">
-        <v>0.3663235888005463</v>
+        <v>0.05395406985361155</v>
       </c>
       <c r="G28" t="n">
-        <v>0.2236158764308646</v>
+        <v>-0.00881187815544715</v>
       </c>
       <c r="H28" t="n">
-        <v>0.1128108501434326</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I28" t="n">
+        <v>0.03188310799021077</v>
+      </c>
+      <c r="J28" t="n">
+        <v>0.7091223558726518</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0.1713425286499376</v>
+      </c>
+      <c r="L28" t="n">
+        <v>0.3316091195362565</v>
+      </c>
+      <c r="M28" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N28" t="n">
+        <v>4.882240772247314</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>MarketCap_sector</t>
+          <t>LASSO_sector</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>125</v>
+        <v>100</v>
       </c>
       <c r="C29" t="n">
-        <v>0.01550250484612793</v>
+        <v>756</v>
       </c>
       <c r="D29" t="n">
-        <v>0.6413996348507045</v>
+        <v>63</v>
       </c>
       <c r="E29" t="n">
-        <v>0.1855234308679941</v>
+        <v>0.03373523188432963</v>
       </c>
       <c r="F29" t="n">
-        <v>0.3692062901810901</v>
+        <v>0.05501290197720669</v>
       </c>
       <c r="G29" t="n">
-        <v>0.2236158764308646</v>
+        <v>-0.008839218068447896</v>
       </c>
       <c r="H29" t="n">
-        <v>0.1586766242980957</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I29" t="n">
+        <v>0.03185576807721002</v>
+      </c>
+      <c r="J29" t="n">
+        <v>0.7065891198678764</v>
+      </c>
+      <c r="K29" t="n">
+        <v>0.0524555268381932</v>
+      </c>
+      <c r="L29" t="n">
+        <v>0.3045587949637398</v>
+      </c>
+      <c r="M29" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N29" t="n">
+        <v>0.3819100856781006</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>LASSO</t>
+          <t>MIQP_Gurobi</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>125</v>
+        <v>100</v>
       </c>
       <c r="C30" t="n">
-        <v>0.01102540564076056</v>
+        <v>756</v>
       </c>
       <c r="D30" t="n">
-        <v>0.5906781594063364</v>
+        <v>63</v>
       </c>
       <c r="E30" t="n">
-        <v>0.3260755340283137</v>
+        <v>0.01274849385010839</v>
       </c>
       <c r="F30" t="n">
-        <v>0.3834720094927412</v>
+        <v>0.02167644004736761</v>
       </c>
       <c r="G30" t="n">
-        <v>0.1822606197395785</v>
+        <v>-0.02009039644168809</v>
       </c>
       <c r="H30" t="n">
-        <v>15.20121216773987</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0.02060458970396983</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0.4637167439201977</v>
+      </c>
+      <c r="K30" t="n">
+        <v>0.1042624566808041</v>
+      </c>
+      <c r="L30" t="n">
+        <v>0.4779760884905953</v>
+      </c>
+      <c r="M30" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N30" t="n">
+        <v>0.8611488342285156</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>LASSO_sector</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>125</v>
+        <v>100</v>
       </c>
       <c r="C31" t="n">
-        <v>0.01270546858248589</v>
+        <v>756</v>
       </c>
       <c r="D31" t="n">
-        <v>0.659091388871254</v>
+        <v>63</v>
       </c>
       <c r="E31" t="n">
-        <v>0.2407053393738546</v>
+        <v>0.0163070889570452</v>
       </c>
       <c r="F31" t="n">
-        <v>0.3790088433424698</v>
+        <v>0.0297896239874123</v>
       </c>
       <c r="G31" t="n">
-        <v>0.1822606197395785</v>
+        <v>-0.02603400114183074</v>
       </c>
       <c r="H31" t="n">
-        <v>14.43701958656311</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0.01466098500382718</v>
+      </c>
+      <c r="J31" t="n">
+        <v>0.5172654599857511</v>
+      </c>
+      <c r="K31" t="n">
+        <v>0.05062078117133128</v>
+      </c>
+      <c r="L31" t="n">
+        <v>0.4349662790494537</v>
+      </c>
+      <c r="M31" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N31" t="n">
+        <v>2.315560579299927</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>MIQP_Gurobi</t>
+          <t>Stratified</t>
         </is>
       </c>
       <c r="B32" t="n">
         <v>125</v>
       </c>
       <c r="C32" t="n">
-        <v>0.01092264746897704</v>
+        <v>756</v>
       </c>
       <c r="D32" t="n">
-        <v>0.6067646074993444</v>
+        <v>63</v>
       </c>
       <c r="E32" t="n">
-        <v>0.3467563591623855</v>
+        <v>0.01501672371542378</v>
       </c>
       <c r="F32" t="n">
-        <v>0.3806957990621284</v>
+        <v>0.02071406052398529</v>
       </c>
       <c r="G32" t="n">
-        <v>0.1745463545501517</v>
+        <v>-0.01969442565401469</v>
       </c>
       <c r="H32" t="n">
-        <v>120.2153079509735</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I32" t="n">
+        <v>0.02100056049164323</v>
+      </c>
+      <c r="J32" t="n">
+        <v>0.4098944381636339</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0.1105206682191056</v>
+      </c>
+      <c r="L32" t="n">
+        <v>0.3611205383047592</v>
+      </c>
+      <c r="M32" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N32" t="n">
+        <v>0.3469243049621582</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Stratified_sector</t>
         </is>
       </c>
       <c r="B33" t="n">
         <v>125</v>
       </c>
       <c r="C33" t="n">
-        <v>0.01598721117287231</v>
+        <v>756</v>
       </c>
       <c r="D33" t="n">
-        <v>0.7393423430476744</v>
+        <v>63</v>
       </c>
       <c r="E33" t="n">
-        <v>0.5098502741288395</v>
+        <v>0.01650219342763259</v>
       </c>
       <c r="F33" t="n">
-        <v>0.3203072206052591</v>
+        <v>0.02536224463272638</v>
       </c>
       <c r="G33" t="n">
-        <v>0.1275419204914943</v>
+        <v>-0.01588560685485907</v>
       </c>
       <c r="H33" t="n">
-        <v>181.4583315849304</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I33" t="n">
+        <v>0.02480937929079885</v>
+      </c>
+      <c r="J33" t="n">
+        <v>0.3976552083315676</v>
+      </c>
+      <c r="K33" t="n">
+        <v>0.03751216589472747</v>
+      </c>
+      <c r="L33" t="n">
+        <v>0.3650172235282855</v>
+      </c>
+      <c r="M33" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N33" t="n">
+        <v>0.5000302791595459</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Stratified</t>
+          <t>MarketCap</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>150</v>
+        <v>125</v>
       </c>
       <c r="C34" t="n">
-        <v>0.01332584813073078</v>
+        <v>756</v>
       </c>
       <c r="D34" t="n">
-        <v>0.6637376571558931</v>
+        <v>63</v>
       </c>
       <c r="E34" t="n">
-        <v>0.292312660311384</v>
+        <v>0.01478096205112091</v>
       </c>
       <c r="F34" t="n">
-        <v>0.3067424008054875</v>
+        <v>0.0192505721710686</v>
       </c>
       <c r="G34" t="n">
-        <v>0.197575295039739</v>
+        <v>-0.01755963613930844</v>
       </c>
       <c r="H34" t="n">
-        <v>0.4722743034362793</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I34" t="n">
+        <v>0.02313535000634948</v>
+      </c>
+      <c r="J34" t="n">
+        <v>0.4106820414758294</v>
+      </c>
+      <c r="K34" t="n">
+        <v>0.1140571186897965</v>
+      </c>
+      <c r="L34" t="n">
+        <v>0.3724430285781953</v>
+      </c>
+      <c r="M34" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N34" t="n">
+        <v>0.2977313995361328</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Stratified_sector</t>
+          <t>MarketCap_sector</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>150</v>
+        <v>125</v>
       </c>
       <c r="C35" t="n">
-        <v>0.01522561190985266</v>
+        <v>756</v>
       </c>
       <c r="D35" t="n">
-        <v>0.6578052035209738</v>
+        <v>63</v>
       </c>
       <c r="E35" t="n">
-        <v>0.1801952434750339</v>
+        <v>0.01622370938578776</v>
       </c>
       <c r="F35" t="n">
-        <v>0.3054147078042637</v>
+        <v>0.02321855967705061</v>
       </c>
       <c r="G35" t="n">
-        <v>0.197575295039739</v>
+        <v>-0.01203755306179821</v>
       </c>
       <c r="H35" t="n">
-        <v>0.8497292995452881</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0.02865743308385971</v>
+      </c>
+      <c r="J35" t="n">
+        <v>0.401642328141955</v>
+      </c>
+      <c r="K35" t="n">
+        <v>0.03970916640621911</v>
+      </c>
+      <c r="L35" t="n">
+        <v>0.3800217018059028</v>
+      </c>
+      <c r="M35" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N35" t="n">
+        <v>0.4234075546264648</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>MarketCap</t>
+          <t>Contribution</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>150</v>
+        <v>125</v>
       </c>
       <c r="C36" t="n">
-        <v>0.013065030784194</v>
+        <v>756</v>
       </c>
       <c r="D36" t="n">
-        <v>0.6685962506988319</v>
+        <v>63</v>
       </c>
       <c r="E36" t="n">
-        <v>0.2817059115526097</v>
+        <v>0.0319657744185568</v>
       </c>
       <c r="F36" t="n">
-        <v>0.3147215195863965</v>
+        <v>0.05449061732302178</v>
       </c>
       <c r="G36" t="n">
-        <v>0.2009106290271965</v>
+        <v>-0.06260012753491129</v>
       </c>
       <c r="H36" t="n">
-        <v>0.5439209938049316</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I36" t="n">
+        <v>-0.02190514138925337</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0.6432338671754387</v>
+      </c>
+      <c r="K36" t="n">
+        <v>0.328554256674129</v>
+      </c>
+      <c r="L36" t="n">
+        <v>0.189728258113615</v>
+      </c>
+      <c r="M36" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N36" t="n">
+        <v>0.2863955497741699</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>MarketCap_sector</t>
+          <t>Contribution_sector</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>150</v>
+        <v>125</v>
       </c>
       <c r="C37" t="n">
-        <v>0.01476957344233265</v>
+        <v>756</v>
       </c>
       <c r="D37" t="n">
-        <v>0.6578385982038568</v>
+        <v>63</v>
       </c>
       <c r="E37" t="n">
-        <v>0.1653806897891988</v>
+        <v>0.04284127173398686</v>
       </c>
       <c r="F37" t="n">
-        <v>0.3164429209950039</v>
+        <v>0.06717370925138769</v>
       </c>
       <c r="G37" t="n">
-        <v>0.2009106290271965</v>
+        <v>-0.06351326569048732</v>
       </c>
       <c r="H37" t="n">
-        <v>0.6826465129852295</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I37" t="n">
+        <v>-0.0228182795448294</v>
+      </c>
+      <c r="J37" t="n">
+        <v>0.6479486722723091</v>
+      </c>
+      <c r="K37" t="n">
+        <v>0.1147599126238575</v>
+      </c>
+      <c r="L37" t="n">
+        <v>0.1706790279798201</v>
+      </c>
+      <c r="M37" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N37" t="n">
+        <v>0.4446251392364502</v>
       </c>
     </row>
     <row r="38">
@@ -1473,25 +2151,43 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>150</v>
+        <v>125</v>
       </c>
       <c r="C38" t="n">
-        <v>0.01078825306808145</v>
+        <v>756</v>
       </c>
       <c r="D38" t="n">
-        <v>0.5700418699197904</v>
+        <v>63</v>
       </c>
       <c r="E38" t="n">
-        <v>0.2814723562243076</v>
+        <v>0.03023761116221356</v>
       </c>
       <c r="F38" t="n">
-        <v>0.3250193677581306</v>
+        <v>0.04699987835918025</v>
       </c>
       <c r="G38" t="n">
-        <v>0.1653960800085443</v>
+        <v>-0.01505539925086563</v>
       </c>
       <c r="H38" t="n">
-        <v>53.72211956977844</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I38" t="n">
+        <v>0.02563958689479229</v>
+      </c>
+      <c r="J38" t="n">
+        <v>0.6849457778951207</v>
+      </c>
+      <c r="K38" t="n">
+        <v>0.1770137365250508</v>
+      </c>
+      <c r="L38" t="n">
+        <v>0.2932748815633798</v>
+      </c>
+      <c r="M38" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N38" t="n">
+        <v>4.354493379592896</v>
       </c>
     </row>
     <row r="39">
@@ -1501,25 +2197,43 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>150</v>
+        <v>125</v>
       </c>
       <c r="C39" t="n">
-        <v>0.01245612482270189</v>
+        <v>756</v>
       </c>
       <c r="D39" t="n">
-        <v>0.6413646957979611</v>
+        <v>63</v>
       </c>
       <c r="E39" t="n">
-        <v>0.2167245135129104</v>
+        <v>0.03212207495462593</v>
       </c>
       <c r="F39" t="n">
-        <v>0.3214668527718408</v>
+        <v>0.0474038227311226</v>
       </c>
       <c r="G39" t="n">
-        <v>0.1653960800085443</v>
+        <v>-0.0156247570722271</v>
       </c>
       <c r="H39" t="n">
-        <v>51.003577709198</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0.02507022907343082</v>
+      </c>
+      <c r="J39" t="n">
+        <v>0.6914322826900101</v>
+      </c>
+      <c r="K39" t="n">
+        <v>0.05572653440477617</v>
+      </c>
+      <c r="L39" t="n">
+        <v>0.262584135562523</v>
+      </c>
+      <c r="M39" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N39" t="n">
+        <v>0.4442825317382812</v>
       </c>
     </row>
     <row r="40">
@@ -1529,25 +2243,43 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>150</v>
+        <v>125</v>
       </c>
       <c r="C40" t="n">
-        <v>0.01079238382940456</v>
+        <v>756</v>
       </c>
       <c r="D40" t="n">
-        <v>0.5738231181294912</v>
+        <v>63</v>
       </c>
       <c r="E40" t="n">
-        <v>0.2810868614162275</v>
+        <v>0.01395781291092483</v>
       </c>
       <c r="F40" t="n">
-        <v>0.3250836045223647</v>
+        <v>0.02565366917621389</v>
       </c>
       <c r="G40" t="n">
-        <v>0.1653463063064307</v>
+        <v>-0.02579455074569814</v>
       </c>
       <c r="H40" t="n">
-        <v>23.36317992210388</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I40" t="n">
+        <v>0.01490043539995978</v>
+      </c>
+      <c r="J40" t="n">
+        <v>0.4768602818672021</v>
+      </c>
+      <c r="K40" t="n">
+        <v>0.1190762089959605</v>
+      </c>
+      <c r="L40" t="n">
+        <v>0.3689654746836568</v>
+      </c>
+      <c r="M40" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N40" t="n">
+        <v>0.959846019744873</v>
       </c>
     </row>
     <row r="41">
@@ -1557,25 +2289,43 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>150</v>
+        <v>125</v>
       </c>
       <c r="C41" t="n">
-        <v>0.01487254308717851</v>
+        <v>756</v>
       </c>
       <c r="D41" t="n">
-        <v>0.7729187972715543</v>
+        <v>63</v>
       </c>
       <c r="E41" t="n">
-        <v>0.484496619048062</v>
+        <v>0.01650968431775742</v>
       </c>
       <c r="F41" t="n">
-        <v>0.272190303858093</v>
+        <v>0.03093588414837352</v>
       </c>
       <c r="G41" t="n">
-        <v>0.1188115480035294</v>
+        <v>-0.0200098835145982</v>
       </c>
       <c r="H41" t="n">
-        <v>181.408616065979</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I41" t="n">
+        <v>0.02068510263105972</v>
+      </c>
+      <c r="J41" t="n">
+        <v>0.4880786765908807</v>
+      </c>
+      <c r="K41" t="n">
+        <v>0.04930478884872755</v>
+      </c>
+      <c r="L41" t="n">
+        <v>0.3583294819886424</v>
+      </c>
+      <c r="M41" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N41" t="n">
+        <v>2.06228232383728</v>
       </c>
     </row>
     <row r="42">
@@ -1585,25 +2335,43 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>175</v>
+        <v>150</v>
       </c>
       <c r="C42" t="n">
-        <v>0.01251459746610982</v>
+        <v>756</v>
       </c>
       <c r="D42" t="n">
-        <v>0.662970322264935</v>
+        <v>63</v>
       </c>
       <c r="E42" t="n">
-        <v>0.2538069006071917</v>
+        <v>0.01438356881926307</v>
       </c>
       <c r="F42" t="n">
-        <v>0.2761691091408736</v>
+        <v>0.02020601788216483</v>
       </c>
       <c r="G42" t="n">
-        <v>0.1812333060481701</v>
+        <v>-0.01918947354078893</v>
       </c>
       <c r="H42" t="n">
-        <v>0.3333828449249268</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I42" t="n">
+        <v>0.02150551260486899</v>
+      </c>
+      <c r="J42" t="n">
+        <v>0.4086198119711728</v>
+      </c>
+      <c r="K42" t="n">
+        <v>0.1061181736197507</v>
+      </c>
+      <c r="L42" t="n">
+        <v>0.3108764604014252</v>
+      </c>
+      <c r="M42" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N42" t="n">
+        <v>0.4930386543273926</v>
       </c>
     </row>
     <row r="43">
@@ -1613,25 +2381,43 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>175</v>
+        <v>150</v>
       </c>
       <c r="C43" t="n">
-        <v>0.01421422074720463</v>
+        <v>756</v>
       </c>
       <c r="D43" t="n">
-        <v>0.675331234502019</v>
+        <v>63</v>
       </c>
       <c r="E43" t="n">
-        <v>0.1580411746412233</v>
+        <v>0.01577590630330238</v>
       </c>
       <c r="F43" t="n">
-        <v>0.2747241457945387</v>
+        <v>0.02420298830023651</v>
       </c>
       <c r="G43" t="n">
-        <v>0.1812333060481701</v>
+        <v>-0.01503055835031497</v>
       </c>
       <c r="H43" t="n">
-        <v>0.4198579788208008</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I43" t="n">
+        <v>0.02566442779534295</v>
+      </c>
+      <c r="J43" t="n">
+        <v>0.3952085099458599</v>
+      </c>
+      <c r="K43" t="n">
+        <v>0.04206727931375008</v>
+      </c>
+      <c r="L43" t="n">
+        <v>0.3151281865258138</v>
+      </c>
+      <c r="M43" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N43" t="n">
+        <v>0.7018122673034668</v>
       </c>
     </row>
     <row r="44">
@@ -1641,25 +2427,43 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>175</v>
+        <v>150</v>
       </c>
       <c r="C44" t="n">
-        <v>0.01250443469876229</v>
+        <v>756</v>
       </c>
       <c r="D44" t="n">
-        <v>0.6621396884794913</v>
+        <v>63</v>
       </c>
       <c r="E44" t="n">
-        <v>0.2575049089407571</v>
+        <v>0.01404612534663762</v>
       </c>
       <c r="F44" t="n">
-        <v>0.2733057848103894</v>
+        <v>0.01909896889094666</v>
       </c>
       <c r="G44" t="n">
-        <v>0.183257428359629</v>
+        <v>-0.01619792698623668</v>
       </c>
       <c r="H44" t="n">
-        <v>0.3754312992095947</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I44" t="n">
+        <v>0.02449705915942124</v>
+      </c>
+      <c r="J44" t="n">
+        <v>0.4003256340272126</v>
+      </c>
+      <c r="K44" t="n">
+        <v>0.110413859766788</v>
+      </c>
+      <c r="L44" t="n">
+        <v>0.3199763824459147</v>
+      </c>
+      <c r="M44" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N44" t="n">
+        <v>0.4163274765014648</v>
       </c>
     </row>
     <row r="45">
@@ -1669,361 +2473,1239 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>175</v>
+        <v>150</v>
       </c>
       <c r="C45" t="n">
-        <v>0.01421061870618985</v>
+        <v>756</v>
       </c>
       <c r="D45" t="n">
-        <v>0.6674657685449747</v>
+        <v>63</v>
       </c>
       <c r="E45" t="n">
-        <v>0.1428385081218448</v>
+        <v>0.01557517091624414</v>
       </c>
       <c r="F45" t="n">
-        <v>0.2737985273557806</v>
+        <v>0.02213740826410911</v>
       </c>
       <c r="G45" t="n">
-        <v>0.183257428359629</v>
+        <v>-0.01152081493252799</v>
       </c>
       <c r="H45" t="n">
-        <v>0.5183541774749756</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0.02917417121312993</v>
+      </c>
+      <c r="J45" t="n">
+        <v>0.3939977254478679</v>
+      </c>
+      <c r="K45" t="n">
+        <v>0.04360154116253735</v>
+      </c>
+      <c r="L45" t="n">
+        <v>0.3246058484494233</v>
+      </c>
+      <c r="M45" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N45" t="n">
+        <v>0.5768575668334961</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>LASSO</t>
+          <t>Contribution</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>175</v>
+        <v>150</v>
       </c>
       <c r="C46" t="n">
-        <v>0.01073414902740281</v>
+        <v>756</v>
       </c>
       <c r="D46" t="n">
-        <v>0.5587854270995692</v>
+        <v>63</v>
       </c>
       <c r="E46" t="n">
-        <v>0.2747749573172037</v>
+        <v>0.02793010186213254</v>
       </c>
       <c r="F46" t="n">
-        <v>0.2820177988138636</v>
+        <v>0.04155464363381731</v>
       </c>
       <c r="G46" t="n">
-        <v>0.1477181451785467</v>
+        <v>-0.05639413185258713</v>
       </c>
       <c r="H46" t="n">
-        <v>22.86103391647339</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I46" t="n">
+        <v>-0.01569914570692921</v>
+      </c>
+      <c r="J46" t="n">
+        <v>0.6316937526271669</v>
+      </c>
+      <c r="K46" t="n">
+        <v>0.276024533126153</v>
+      </c>
+      <c r="L46" t="n">
+        <v>0.1595161058683227</v>
+      </c>
+      <c r="M46" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N46" t="n">
+        <v>0.4301791191101074</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>LASSO_sector</t>
+          <t>Contribution_sector</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>175</v>
+        <v>150</v>
       </c>
       <c r="C47" t="n">
-        <v>0.01220176333553115</v>
+        <v>756</v>
       </c>
       <c r="D47" t="n">
-        <v>0.6296697773601843</v>
+        <v>63</v>
       </c>
       <c r="E47" t="n">
-        <v>0.218774525000247</v>
+        <v>0.03399702959548037</v>
       </c>
       <c r="F47" t="n">
-        <v>0.2803928588670065</v>
+        <v>0.04612788168830206</v>
       </c>
       <c r="G47" t="n">
-        <v>0.1477181451785467</v>
+        <v>-0.06072876215926915</v>
       </c>
       <c r="H47" t="n">
-        <v>22.47959971427917</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I47" t="n">
+        <v>-0.02003377601361123</v>
+      </c>
+      <c r="J47" t="n">
+        <v>0.6349259357217522</v>
+      </c>
+      <c r="K47" t="n">
+        <v>0.1147599126238575</v>
+      </c>
+      <c r="L47" t="n">
+        <v>0.1667532518400083</v>
+      </c>
+      <c r="M47" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N47" t="n">
+        <v>0.7087323665618896</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>MIQP_Gurobi</t>
+          <t>LASSO</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>175</v>
+        <v>150</v>
       </c>
       <c r="C48" t="n">
-        <v>0.01079075850996434</v>
+        <v>756</v>
       </c>
       <c r="D48" t="n">
-        <v>0.5659185357959817</v>
+        <v>63</v>
       </c>
       <c r="E48" t="n">
-        <v>0.2728075362318651</v>
+        <v>0.02834588913380612</v>
       </c>
       <c r="F48" t="n">
-        <v>0.2816908159475793</v>
+        <v>0.04353047940382004</v>
       </c>
       <c r="G48" t="n">
-        <v>0.1474341558916836</v>
+        <v>-0.01754339711571529</v>
       </c>
       <c r="H48" t="n">
-        <v>6.256840467453003</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I48" t="n">
+        <v>0.02315158902994263</v>
+      </c>
+      <c r="J48" t="n">
+        <v>0.650068729060665</v>
+      </c>
+      <c r="K48" t="n">
+        <v>0.1862597558528913</v>
+      </c>
+      <c r="L48" t="n">
+        <v>0.2562950217268639</v>
+      </c>
+      <c r="M48" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N48" t="n">
+        <v>7.164833068847656</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>LASSO_sector</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>175</v>
+        <v>150</v>
       </c>
       <c r="C49" t="n">
-        <v>0.01356002319023514</v>
+        <v>756</v>
       </c>
       <c r="D49" t="n">
-        <v>0.7001473545696448</v>
+        <v>63</v>
       </c>
       <c r="E49" t="n">
-        <v>0.3982880909414317</v>
+        <v>0.03041429943670386</v>
       </c>
       <c r="F49" t="n">
-        <v>0.2547141103823961</v>
+        <v>0.04643243399260925</v>
       </c>
       <c r="G49" t="n">
-        <v>0.1123680419409523</v>
+        <v>-0.01362387012923949</v>
       </c>
       <c r="H49" t="n">
-        <v>181.9129874706268</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I49" t="n">
+        <v>0.02707111601641843</v>
+      </c>
+      <c r="J49" t="n">
+        <v>0.6628935955305592</v>
+      </c>
+      <c r="K49" t="n">
+        <v>0.0523721919427817</v>
+      </c>
+      <c r="L49" t="n">
+        <v>0.2446414102039493</v>
+      </c>
+      <c r="M49" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N49" t="n">
+        <v>0.667339563369751</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Stratified</t>
+          <t>MIQP_Gurobi</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="C50" t="n">
-        <v>0.01238842601907632</v>
+        <v>756</v>
       </c>
       <c r="D50" t="n">
-        <v>0.6633644956739029</v>
+        <v>63</v>
       </c>
       <c r="E50" t="n">
-        <v>0.2366200390728226</v>
+        <v>0.01538875837345898</v>
       </c>
       <c r="F50" t="n">
-        <v>0.2433341107305037</v>
+        <v>0.02546786834069736</v>
       </c>
       <c r="G50" t="n">
-        <v>0.1668723001381942</v>
+        <v>-0.0153711702320708</v>
       </c>
       <c r="H50" t="n">
-        <v>1.01370906829834</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I50" t="n">
+        <v>0.02532381591358712</v>
+      </c>
+      <c r="J50" t="n">
+        <v>0.4863301727866063</v>
+      </c>
+      <c r="K50" t="n">
+        <v>0.1066342991865511</v>
+      </c>
+      <c r="L50" t="n">
+        <v>0.307193873387</v>
+      </c>
+      <c r="M50" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N50" t="n">
+        <v>1.134274005889893</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Stratified_sector</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="C51" t="n">
-        <v>0.01402369603105219</v>
+        <v>756</v>
       </c>
       <c r="D51" t="n">
-        <v>0.678252240510574</v>
+        <v>63</v>
       </c>
       <c r="E51" t="n">
-        <v>0.1383558030646831</v>
+        <v>0.01670858041203334</v>
       </c>
       <c r="F51" t="n">
-        <v>0.2421509390425457</v>
+        <v>0.02906381070400115</v>
       </c>
       <c r="G51" t="n">
-        <v>0.1668723001381942</v>
+        <v>-0.006906314888562193</v>
       </c>
       <c r="H51" t="n">
-        <v>1.808587074279785</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I51" t="n">
+        <v>0.03378867125709573</v>
+      </c>
+      <c r="J51" t="n">
+        <v>0.4889272151710584</v>
+      </c>
+      <c r="K51" t="n">
+        <v>0.04002563731453083</v>
+      </c>
+      <c r="L51" t="n">
+        <v>0.3107997003392006</v>
+      </c>
+      <c r="M51" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N51" t="n">
+        <v>1.788345336914062</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>MarketCap</t>
+          <t>Stratified</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>200</v>
+        <v>175</v>
       </c>
       <c r="C52" t="n">
-        <v>0.01217545982067404</v>
+        <v>756</v>
       </c>
       <c r="D52" t="n">
-        <v>0.6602749432290103</v>
+        <v>63</v>
       </c>
       <c r="E52" t="n">
-        <v>0.227080656039524</v>
+        <v>0.01373659029515908</v>
       </c>
       <c r="F52" t="n">
-        <v>0.2405637704844487</v>
+        <v>0.01952093978617634</v>
       </c>
       <c r="G52" t="n">
-        <v>0.1685071143976193</v>
+        <v>-0.01546598142159306</v>
       </c>
       <c r="H52" t="n">
-        <v>1.145128726959229</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I52" t="n">
+        <v>0.02522900472406486</v>
+      </c>
+      <c r="J52" t="n">
+        <v>0.4016785416600893</v>
+      </c>
+      <c r="K52" t="n">
+        <v>0.1031687690517409</v>
+      </c>
+      <c r="L52" t="n">
+        <v>0.275242341209694</v>
+      </c>
+      <c r="M52" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N52" t="n">
+        <v>0.5624418258666992</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>MarketCap_sector</t>
+          <t>Stratified_sector</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>200</v>
+        <v>175</v>
       </c>
       <c r="C53" t="n">
-        <v>0.01379778958304354</v>
+        <v>756</v>
       </c>
       <c r="D53" t="n">
-        <v>0.6869573151639125</v>
+        <v>63</v>
       </c>
       <c r="E53" t="n">
-        <v>0.1207176247935243</v>
+        <v>0.01517153618584891</v>
       </c>
       <c r="F53" t="n">
-        <v>0.2394771244044434</v>
+        <v>0.02282747197253459</v>
       </c>
       <c r="G53" t="n">
-        <v>0.1685071143976193</v>
+        <v>-0.009461683543367183</v>
       </c>
       <c r="H53" t="n">
-        <v>1.449644327163696</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I53" t="n">
+        <v>0.03123330260229074</v>
+      </c>
+      <c r="J53" t="n">
+        <v>0.3946867050923578</v>
+      </c>
+      <c r="K53" t="n">
+        <v>0.0409388467230196</v>
+      </c>
+      <c r="L53" t="n">
+        <v>0.277130032520464</v>
+      </c>
+      <c r="M53" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N53" t="n">
+        <v>0.7294037342071533</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>LASSO</t>
+          <t>MarketCap</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>200</v>
+        <v>175</v>
       </c>
       <c r="C54" t="n">
-        <v>0.01072880028499942</v>
+        <v>756</v>
       </c>
       <c r="D54" t="n">
-        <v>0.5667402591613868</v>
+        <v>63</v>
       </c>
       <c r="E54" t="n">
-        <v>0.2512469863395484</v>
+        <v>0.01353855154535205</v>
       </c>
       <c r="F54" t="n">
-        <v>0.2475010482313282</v>
+        <v>0.018644162000766</v>
       </c>
       <c r="G54" t="n">
-        <v>0.1382350828648889</v>
+        <v>-0.01450676628165881</v>
       </c>
       <c r="H54" t="n">
-        <v>57.18866896629333</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I54" t="n">
+        <v>0.02618821986399911</v>
+      </c>
+      <c r="J54" t="n">
+        <v>0.4056626274754821</v>
+      </c>
+      <c r="K54" t="n">
+        <v>0.1037356030755694</v>
+      </c>
+      <c r="L54" t="n">
+        <v>0.2774056312145676</v>
+      </c>
+      <c r="M54" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N54" t="n">
+        <v>0.5068333148956299</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>LASSO_sector</t>
+          <t>MarketCap_sector</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>200</v>
+        <v>175</v>
       </c>
       <c r="C55" t="n">
-        <v>0.01207103731844568</v>
+        <v>756</v>
       </c>
       <c r="D55" t="n">
-        <v>0.6297901382082678</v>
+        <v>63</v>
       </c>
       <c r="E55" t="n">
-        <v>0.204965631461027</v>
+        <v>0.01496589872692473</v>
       </c>
       <c r="F55" t="n">
-        <v>0.246787770215918</v>
+        <v>0.0221683530744774</v>
       </c>
       <c r="G55" t="n">
-        <v>0.1382350828648889</v>
+        <v>-0.009485152373497452</v>
       </c>
       <c r="H55" t="n">
-        <v>57.42676472663879</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I55" t="n">
+        <v>0.03120983377216047</v>
+      </c>
+      <c r="J55" t="n">
+        <v>0.3995172097814074</v>
+      </c>
+      <c r="K55" t="n">
+        <v>0.03910987414901393</v>
+      </c>
+      <c r="L55" t="n">
+        <v>0.2785177962368729</v>
+      </c>
+      <c r="M55" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N55" t="n">
+        <v>0.7753665447235107</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>MIQP_Gurobi</t>
+          <t>Contribution</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>200</v>
+        <v>175</v>
       </c>
       <c r="C56" t="n">
-        <v>0.01074553347222126</v>
+        <v>756</v>
       </c>
       <c r="D56" t="n">
-        <v>0.5707374115858561</v>
+        <v>63</v>
       </c>
       <c r="E56" t="n">
-        <v>0.2539186321810637</v>
+        <v>0.02667355914952692</v>
       </c>
       <c r="F56" t="n">
-        <v>0.2471732841570914</v>
+        <v>0.03657061863375772</v>
       </c>
       <c r="G56" t="n">
-        <v>0.1375093519976635</v>
+        <v>-0.04628114686245099</v>
       </c>
       <c r="H56" t="n">
-        <v>2.972833871841431</v>
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I56" t="n">
+        <v>-0.005586160716793076</v>
+      </c>
+      <c r="J56" t="n">
+        <v>0.6197368431314264</v>
+      </c>
+      <c r="K56" t="n">
+        <v>0.2771236033485901</v>
+      </c>
+      <c r="L56" t="n">
+        <v>0.1528894681421784</v>
+      </c>
+      <c r="M56" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N56" t="n">
+        <v>0.5135312080383301</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
+          <t>Contribution_sector</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>175</v>
+      </c>
+      <c r="C57" t="n">
+        <v>756</v>
+      </c>
+      <c r="D57" t="n">
+        <v>63</v>
+      </c>
+      <c r="E57" t="n">
+        <v>0.03349823606637661</v>
+      </c>
+      <c r="F57" t="n">
+        <v>0.04508335649798993</v>
+      </c>
+      <c r="G57" t="n">
+        <v>-0.0617193966143027</v>
+      </c>
+      <c r="H57" t="n">
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I57" t="n">
+        <v>-0.02102441046864478</v>
+      </c>
+      <c r="J57" t="n">
+        <v>0.6322754140274465</v>
+      </c>
+      <c r="K57" t="n">
+        <v>0.09342960333875344</v>
+      </c>
+      <c r="L57" t="n">
+        <v>0.1492423860285111</v>
+      </c>
+      <c r="M57" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N57" t="n">
+        <v>0.8172359466552734</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>LASSO</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>175</v>
+      </c>
+      <c r="C58" t="n">
+        <v>756</v>
+      </c>
+      <c r="D58" t="n">
+        <v>63</v>
+      </c>
+      <c r="E58" t="n">
+        <v>0.02745369575285448</v>
+      </c>
+      <c r="F58" t="n">
+        <v>0.04054878383551472</v>
+      </c>
+      <c r="G58" t="n">
+        <v>-0.01206490358760282</v>
+      </c>
+      <c r="H58" t="n">
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I58" t="n">
+        <v>0.0286300825580551</v>
+      </c>
+      <c r="J58" t="n">
+        <v>0.6393718574591989</v>
+      </c>
+      <c r="K58" t="n">
+        <v>0.1902547018015324</v>
+      </c>
+      <c r="L58" t="n">
+        <v>0.225854676858655</v>
+      </c>
+      <c r="M58" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N58" t="n">
+        <v>4.507211446762085</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>LASSO_sector</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>175</v>
+      </c>
+      <c r="C59" t="n">
+        <v>756</v>
+      </c>
+      <c r="D59" t="n">
+        <v>63</v>
+      </c>
+      <c r="E59" t="n">
+        <v>0.02972095355061422</v>
+      </c>
+      <c r="F59" t="n">
+        <v>0.04505474506702138</v>
+      </c>
+      <c r="G59" t="n">
+        <v>-0.009826654453622963</v>
+      </c>
+      <c r="H59" t="n">
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I59" t="n">
+        <v>0.03086833169203496</v>
+      </c>
+      <c r="J59" t="n">
+        <v>0.6517119955053394</v>
+      </c>
+      <c r="K59" t="n">
+        <v>0.0523493947513124</v>
+      </c>
+      <c r="L59" t="n">
+        <v>0.2132822122839352</v>
+      </c>
+      <c r="M59" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N59" t="n">
+        <v>0.8197300434112549</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>MIQP_Gurobi</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>175</v>
+      </c>
+      <c r="C60" t="n">
+        <v>756</v>
+      </c>
+      <c r="D60" t="n">
+        <v>63</v>
+      </c>
+      <c r="E60" t="n">
+        <v>0.01469353378213398</v>
+      </c>
+      <c r="F60" t="n">
+        <v>0.02560256636505499</v>
+      </c>
+      <c r="G60" t="n">
+        <v>-0.01748824862099407</v>
+      </c>
+      <c r="H60" t="n">
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I60" t="n">
+        <v>0.02320673752466385</v>
+      </c>
+      <c r="J60" t="n">
+        <v>0.468320494220609</v>
+      </c>
+      <c r="K60" t="n">
+        <v>0.1020931655277634</v>
+      </c>
+      <c r="L60" t="n">
+        <v>0.273431838766101</v>
+      </c>
+      <c r="M60" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N60" t="n">
+        <v>1.243364095687866</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
           <t>Layered</t>
         </is>
       </c>
-      <c r="B57" t="n">
+      <c r="B61" t="n">
+        <v>175</v>
+      </c>
+      <c r="C61" t="n">
+        <v>756</v>
+      </c>
+      <c r="D61" t="n">
+        <v>63</v>
+      </c>
+      <c r="E61" t="n">
+        <v>0.01569773482049812</v>
+      </c>
+      <c r="F61" t="n">
+        <v>0.02526505065716036</v>
+      </c>
+      <c r="G61" t="n">
+        <v>-0.01282507306477487</v>
+      </c>
+      <c r="H61" t="n">
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I61" t="n">
+        <v>0.02786991308088305</v>
+      </c>
+      <c r="J61" t="n">
+        <v>0.4575896632794935</v>
+      </c>
+      <c r="K61" t="n">
+        <v>0.04413284046267384</v>
+      </c>
+      <c r="L61" t="n">
+        <v>0.2769434147089305</v>
+      </c>
+      <c r="M61" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N61" t="n">
+        <v>1.597336769104004</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Stratified</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
         <v>200</v>
       </c>
-      <c r="C57" t="n">
-        <v>0.01322924844333005</v>
-      </c>
-      <c r="D57" t="n">
-        <v>0.7316004259728994</v>
-      </c>
-      <c r="E57" t="n">
-        <v>0.4251411323529834</v>
-      </c>
-      <c r="F57" t="n">
-        <v>0.2162557174708556</v>
-      </c>
-      <c r="G57" t="n">
-        <v>0.1027397627438593</v>
-      </c>
-      <c r="H57" t="n">
-        <v>181.6314015388489</v>
+      <c r="C62" t="n">
+        <v>756</v>
+      </c>
+      <c r="D62" t="n">
+        <v>63</v>
+      </c>
+      <c r="E62" t="n">
+        <v>0.01345106671728012</v>
+      </c>
+      <c r="F62" t="n">
+        <v>0.019117613269477</v>
+      </c>
+      <c r="G62" t="n">
+        <v>-0.01555786674780602</v>
+      </c>
+      <c r="H62" t="n">
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I62" t="n">
+        <v>0.0251371193978519</v>
+      </c>
+      <c r="J62" t="n">
+        <v>0.3994951507063763</v>
+      </c>
+      <c r="K62" t="n">
+        <v>0.1039892877439424</v>
+      </c>
+      <c r="L62" t="n">
+        <v>0.2469977988333879</v>
+      </c>
+      <c r="M62" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N62" t="n">
+        <v>0.6461918354034424</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Stratified_sector</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>200</v>
+      </c>
+      <c r="C63" t="n">
+        <v>756</v>
+      </c>
+      <c r="D63" t="n">
+        <v>63</v>
+      </c>
+      <c r="E63" t="n">
+        <v>0.01491821657578082</v>
+      </c>
+      <c r="F63" t="n">
+        <v>0.02225112933277049</v>
+      </c>
+      <c r="G63" t="n">
+        <v>-0.01023017324162878</v>
+      </c>
+      <c r="H63" t="n">
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I63" t="n">
+        <v>0.03046481290402914</v>
+      </c>
+      <c r="J63" t="n">
+        <v>0.3929238476953178</v>
+      </c>
+      <c r="K63" t="n">
+        <v>0.03715893409147148</v>
+      </c>
+      <c r="L63" t="n">
+        <v>0.2478533418551931</v>
+      </c>
+      <c r="M63" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N63" t="n">
+        <v>1.025138378143311</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>MarketCap</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>200</v>
+      </c>
+      <c r="C64" t="n">
+        <v>756</v>
+      </c>
+      <c r="D64" t="n">
+        <v>63</v>
+      </c>
+      <c r="E64" t="n">
+        <v>0.01331263935425953</v>
+      </c>
+      <c r="F64" t="n">
+        <v>0.01898524165220005</v>
+      </c>
+      <c r="G64" t="n">
+        <v>-0.01498674724447813</v>
+      </c>
+      <c r="H64" t="n">
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I64" t="n">
+        <v>0.02570823890117979</v>
+      </c>
+      <c r="J64" t="n">
+        <v>0.3975591241939296</v>
+      </c>
+      <c r="K64" t="n">
+        <v>0.1005137994954309</v>
+      </c>
+      <c r="L64" t="n">
+        <v>0.2477412851561393</v>
+      </c>
+      <c r="M64" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N64" t="n">
+        <v>0.6550312042236328</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>MarketCap_sector</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>200</v>
+      </c>
+      <c r="C65" t="n">
+        <v>756</v>
+      </c>
+      <c r="D65" t="n">
+        <v>63</v>
+      </c>
+      <c r="E65" t="n">
+        <v>0.01445491782964153</v>
+      </c>
+      <c r="F65" t="n">
+        <v>0.02130139122366886</v>
+      </c>
+      <c r="G65" t="n">
+        <v>-0.01178810825568044</v>
+      </c>
+      <c r="H65" t="n">
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I65" t="n">
+        <v>0.02890687788997748</v>
+      </c>
+      <c r="J65" t="n">
+        <v>0.3946629826653786</v>
+      </c>
+      <c r="K65" t="n">
+        <v>0.03862999255173426</v>
+      </c>
+      <c r="L65" t="n">
+        <v>0.2491293132665541</v>
+      </c>
+      <c r="M65" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N65" t="n">
+        <v>0.944951057434082</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Contribution</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>200</v>
+      </c>
+      <c r="C66" t="n">
+        <v>756</v>
+      </c>
+      <c r="D66" t="n">
+        <v>63</v>
+      </c>
+      <c r="E66" t="n">
+        <v>0.02394882832963548</v>
+      </c>
+      <c r="F66" t="n">
+        <v>0.02887828711992035</v>
+      </c>
+      <c r="G66" t="n">
+        <v>-0.02544879408933687</v>
+      </c>
+      <c r="H66" t="n">
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I66" t="n">
+        <v>0.01524619205632105</v>
+      </c>
+      <c r="J66" t="n">
+        <v>0.5962512092394441</v>
+      </c>
+      <c r="K66" t="n">
+        <v>0.1866730671088996</v>
+      </c>
+      <c r="L66" t="n">
+        <v>0.1556407863440069</v>
+      </c>
+      <c r="M66" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N66" t="n">
+        <v>0.7366149425506592</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Contribution_sector</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>200</v>
+      </c>
+      <c r="C67" t="n">
+        <v>756</v>
+      </c>
+      <c r="D67" t="n">
+        <v>63</v>
+      </c>
+      <c r="E67" t="n">
+        <v>0.02709773661506483</v>
+      </c>
+      <c r="F67" t="n">
+        <v>0.0306497071631268</v>
+      </c>
+      <c r="G67" t="n">
+        <v>-0.02286211957590711</v>
+      </c>
+      <c r="H67" t="n">
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I67" t="n">
+        <v>0.0178328665697508</v>
+      </c>
+      <c r="J67" t="n">
+        <v>0.6039057214427401</v>
+      </c>
+      <c r="K67" t="n">
+        <v>0.04772216547852231</v>
+      </c>
+      <c r="L67" t="n">
+        <v>0.1506838575649845</v>
+      </c>
+      <c r="M67" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N67" t="n">
+        <v>1.049088716506958</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>LASSO</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>200</v>
+      </c>
+      <c r="C68" t="n">
+        <v>756</v>
+      </c>
+      <c r="D68" t="n">
+        <v>63</v>
+      </c>
+      <c r="E68" t="n">
+        <v>0.02140650039369774</v>
+      </c>
+      <c r="F68" t="n">
+        <v>0.02806881612557981</v>
+      </c>
+      <c r="G68" t="n">
+        <v>-0.008098070681547664</v>
+      </c>
+      <c r="H68" t="n">
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I68" t="n">
+        <v>0.03259691546411025</v>
+      </c>
+      <c r="J68" t="n">
+        <v>0.5718211171670677</v>
+      </c>
+      <c r="K68" t="n">
+        <v>0.1545652775129592</v>
+      </c>
+      <c r="L68" t="n">
+        <v>0.1927267880255058</v>
+      </c>
+      <c r="M68" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N68" t="n">
+        <v>5.430041074752808</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>LASSO_sector</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>200</v>
+      </c>
+      <c r="C69" t="n">
+        <v>756</v>
+      </c>
+      <c r="D69" t="n">
+        <v>63</v>
+      </c>
+      <c r="E69" t="n">
+        <v>0.02403799263573617</v>
+      </c>
+      <c r="F69" t="n">
+        <v>0.03272457676373729</v>
+      </c>
+      <c r="G69" t="n">
+        <v>0.003185494836098757</v>
+      </c>
+      <c r="H69" t="n">
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I69" t="n">
+        <v>0.04388048098175668</v>
+      </c>
+      <c r="J69" t="n">
+        <v>0.5785580168572503</v>
+      </c>
+      <c r="K69" t="n">
+        <v>0.04452949095985319</v>
+      </c>
+      <c r="L69" t="n">
+        <v>0.1944588518847036</v>
+      </c>
+      <c r="M69" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N69" t="n">
+        <v>1.035216093063354</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>MIQP_Gurobi</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>200</v>
+      </c>
+      <c r="C70" t="n">
+        <v>756</v>
+      </c>
+      <c r="D70" t="n">
+        <v>63</v>
+      </c>
+      <c r="E70" t="n">
+        <v>0.01197069458674844</v>
+      </c>
+      <c r="F70" t="n">
+        <v>0.02185997377080254</v>
+      </c>
+      <c r="G70" t="n">
+        <v>-0.02338222653186361</v>
+      </c>
+      <c r="H70" t="n">
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I70" t="n">
+        <v>0.0173127596137943</v>
+      </c>
+      <c r="J70" t="n">
+        <v>0.4051940772552043</v>
+      </c>
+      <c r="K70" t="n">
+        <v>0.1052340913503186</v>
+      </c>
+      <c r="L70" t="n">
+        <v>0.2576277197172963</v>
+      </c>
+      <c r="M70" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N70" t="n">
+        <v>1.173588991165161</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Layered</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>200</v>
+      </c>
+      <c r="C71" t="n">
+        <v>756</v>
+      </c>
+      <c r="D71" t="n">
+        <v>63</v>
+      </c>
+      <c r="E71" t="n">
+        <v>0.01288654450782975</v>
+      </c>
+      <c r="F71" t="n">
+        <v>0.02329015121170905</v>
+      </c>
+      <c r="G71" t="n">
+        <v>-0.0204803197216058</v>
+      </c>
+      <c r="H71" t="n">
+        <v>-0.04069498614565792</v>
+      </c>
+      <c r="I71" t="n">
+        <v>0.02021466642405212</v>
+      </c>
+      <c r="J71" t="n">
+        <v>0.4014893433616881</v>
+      </c>
+      <c r="K71" t="n">
+        <v>0.04665456779454845</v>
+      </c>
+      <c r="L71" t="n">
+        <v>0.2635995786502407</v>
+      </c>
+      <c r="M71" t="n">
+        <v>0.09034232650304058</v>
+      </c>
+      <c r="N71" t="n">
+        <v>1.875100612640381</v>
       </c>
     </row>
   </sheetData>

</xml_diff>